<commit_message>
Added Unit Description tab to the main schema file.
</commit_message>
<xml_diff>
--- a/docs/CDOP_SCHEMA.xlsx
+++ b/docs/CDOP_SCHEMA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ghoffman\Other-GitHub\Carbon-Data-Open-Protocol\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nikodem_lacki/Documents/work/Carbon-Data-Open-Protocol/Carbon-Data-Open-Protocol/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A21B714A-6CD9-4FF5-A0BA-B8A575A27B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB2C76EC-64A6-094D-8D1D-959D7E8DB494}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{743398AF-A4FE-47C4-9368-972E95242EBF}"/>
+    <workbookView xWindow="1320" yWindow="600" windowWidth="33940" windowHeight="15180" activeTab="5" xr2:uid="{743398AF-A4FE-47C4-9368-972E95242EBF}"/>
   </bookViews>
   <sheets>
     <sheet name="Full List" sheetId="5" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="Project Approach &amp; Details" sheetId="2" r:id="rId3"/>
     <sheet name="Issuances" sheetId="3" r:id="rId4"/>
     <sheet name="Disclosures" sheetId="4" r:id="rId5"/>
+    <sheet name="Unit Description" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3184" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3350" uniqueCount="354">
   <si>
     <t>schema</t>
   </si>
@@ -988,6 +989,120 @@
   </si>
   <si>
     <t>list of attestations (e.g., child labor, labor worker attestation), if verified credentials are supported</t>
+  </si>
+  <si>
+    <t>current registry project id</t>
+  </si>
+  <si>
+    <t>Project</t>
+  </si>
+  <si>
+    <t>Registry</t>
+  </si>
+  <si>
+    <t>Identifier used to track the project in the current registry.</t>
+  </si>
+  <si>
+    <t>metric</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Project developer</t>
+  </si>
+  <si>
+    <t>Unit of measurment for quantifying the reduction or removal</t>
+  </si>
+  <si>
+    <t>owner account id</t>
+  </si>
+  <si>
+    <t>GUID</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>identifier for the owner of the unit</t>
+  </si>
+  <si>
+    <t>retirement beneficiary</t>
+  </si>
+  <si>
+    <t>Entity name on behalf of which the retirement occurred</t>
+  </si>
+  <si>
+    <t>retirement detail</t>
+  </si>
+  <si>
+    <t>Additional context describing the retirements</t>
+  </si>
+  <si>
+    <t>serial number</t>
+  </si>
+  <si>
+    <t>Serial number of the unit</t>
+  </si>
+  <si>
+    <t>source serial number</t>
+  </si>
+  <si>
+    <t>Identifier used to track the unit to the original issuance it was part of.</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>Unit state, indicating which lifecycle the unit is currently in</t>
+  </si>
+  <si>
+    <t>status reason</t>
+  </si>
+  <si>
+    <t>String</t>
+  </si>
+  <si>
+    <t>User Input</t>
+  </si>
+  <si>
+    <t>Select the status that best desribes the current state of the units.</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>Descirbes the type of unit.</t>
+  </si>
+  <si>
+    <t>quantity</t>
+  </si>
+  <si>
+    <t>Quantity of units included in the credit block that a particular record represents</t>
+  </si>
+  <si>
+    <t>block end</t>
+  </si>
+  <si>
+    <t>Carbon Crediting Program/ Standard Setters</t>
+  </si>
+  <si>
+    <t>Number indicating the last unit within a credit block</t>
+  </si>
+  <si>
+    <t>block start</t>
+  </si>
+  <si>
+    <t>Number indicating the first unit within a credit block</t>
+  </si>
+  <si>
+    <t>vintage</t>
+  </si>
+  <si>
+    <t>Vintage</t>
+  </si>
+  <si>
+    <t>Temporal period when the envrionmental benefit occurred</t>
   </si>
 </sst>
 </file>
@@ -1493,22 +1608,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{752D3095-90A4-45FF-BD20-0492A3C6EFAC}">
   <dimension ref="A1:L143"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="21.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.77734375" customWidth="1"/>
+    <col min="2" max="2" width="21.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.83203125" customWidth="1"/>
     <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.44140625" customWidth="1"/>
-    <col min="8" max="8" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5" customWidth="1"/>
+    <col min="8" max="8" width="17.5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="25" customWidth="1"/>
-    <col min="10" max="10" width="12.21875" customWidth="1"/>
-    <col min="11" max="11" width="14.21875" customWidth="1"/>
+    <col min="10" max="10" width="12.1640625" customWidth="1"/>
+    <col min="11" max="11" width="14.1640625" customWidth="1"/>
     <col min="12" max="12" width="88" customWidth="1"/>
-    <col min="13" max="18" width="9.21875" customWidth="1"/>
+    <col min="13" max="18" width="9.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1546,7 +1661,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -1584,7 +1699,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1622,7 +1737,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1660,7 +1775,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1698,7 +1813,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1736,7 +1851,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1774,7 +1889,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -1812,7 +1927,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -1850,7 +1965,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -1888,7 +2003,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -1926,7 +2041,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -1964,7 +2079,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -2002,7 +2117,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -2040,7 +2155,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -2078,7 +2193,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>12</v>
       </c>
@@ -2116,7 +2231,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>12</v>
       </c>
@@ -2154,7 +2269,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>12</v>
       </c>
@@ -2192,7 +2307,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>12</v>
       </c>
@@ -2230,7 +2345,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -2268,7 +2383,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>12</v>
       </c>
@@ -2306,7 +2421,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>12</v>
       </c>
@@ -2344,7 +2459,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>12</v>
       </c>
@@ -2382,7 +2497,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>12</v>
       </c>
@@ -2420,7 +2535,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -2458,7 +2573,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>12</v>
       </c>
@@ -2496,7 +2611,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>12</v>
       </c>
@@ -2534,7 +2649,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>12</v>
       </c>
@@ -2572,7 +2687,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>12</v>
       </c>
@@ -2610,7 +2725,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>12</v>
       </c>
@@ -2648,7 +2763,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>12</v>
       </c>
@@ -2686,7 +2801,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>12</v>
       </c>
@@ -2724,7 +2839,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>12</v>
       </c>
@@ -2762,7 +2877,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>12</v>
       </c>
@@ -2800,7 +2915,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>12</v>
       </c>
@@ -2838,7 +2953,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>12</v>
       </c>
@@ -2876,7 +2991,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>12</v>
       </c>
@@ -2914,7 +3029,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>12</v>
       </c>
@@ -2952,7 +3067,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>12</v>
       </c>
@@ -2990,7 +3105,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>12</v>
       </c>
@@ -3028,7 +3143,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>12</v>
       </c>
@@ -3066,7 +3181,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>12</v>
       </c>
@@ -3104,7 +3219,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>12</v>
       </c>
@@ -3142,7 +3257,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>12</v>
       </c>
@@ -3180,7 +3295,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>12</v>
       </c>
@@ -3218,7 +3333,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>12</v>
       </c>
@@ -3256,7 +3371,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>12</v>
       </c>
@@ -3294,7 +3409,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>12</v>
       </c>
@@ -3332,7 +3447,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>12</v>
       </c>
@@ -3370,7 +3485,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>12</v>
       </c>
@@ -3408,7 +3523,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>12</v>
       </c>
@@ -3446,7 +3561,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>12</v>
       </c>
@@ -3484,7 +3599,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>12</v>
       </c>
@@ -3522,7 +3637,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>12</v>
       </c>
@@ -3560,7 +3675,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>12</v>
       </c>
@@ -3598,7 +3713,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>12</v>
       </c>
@@ -3636,7 +3751,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>12</v>
       </c>
@@ -3674,7 +3789,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>12</v>
       </c>
@@ -3712,7 +3827,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>12</v>
       </c>
@@ -3750,7 +3865,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>12</v>
       </c>
@@ -3788,7 +3903,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>12</v>
       </c>
@@ -3826,7 +3941,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>12</v>
       </c>
@@ -3864,7 +3979,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>12</v>
       </c>
@@ -3902,7 +4017,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>12</v>
       </c>
@@ -3940,7 +4055,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>12</v>
       </c>
@@ -3978,7 +4093,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>12</v>
       </c>
@@ -4016,7 +4131,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>12</v>
       </c>
@@ -4054,7 +4169,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>12</v>
       </c>
@@ -4092,7 +4207,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>12</v>
       </c>
@@ -4130,7 +4245,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>12</v>
       </c>
@@ -4168,7 +4283,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>12</v>
       </c>
@@ -4206,7 +4321,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>12</v>
       </c>
@@ -4244,7 +4359,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>12</v>
       </c>
@@ -4282,7 +4397,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>12</v>
       </c>
@@ -4320,7 +4435,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>12</v>
       </c>
@@ -4358,7 +4473,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>12</v>
       </c>
@@ -4396,7 +4511,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>12</v>
       </c>
@@ -4434,7 +4549,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>12</v>
       </c>
@@ -4472,7 +4587,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>12</v>
       </c>
@@ -4510,7 +4625,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>12</v>
       </c>
@@ -4548,7 +4663,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>12</v>
       </c>
@@ -4586,7 +4701,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>12</v>
       </c>
@@ -4624,7 +4739,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>12</v>
       </c>
@@ -4662,7 +4777,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>12</v>
       </c>
@@ -4700,7 +4815,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>12</v>
       </c>
@@ -4738,7 +4853,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>12</v>
       </c>
@@ -4776,7 +4891,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>12</v>
       </c>
@@ -4814,7 +4929,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>12</v>
       </c>
@@ -4852,7 +4967,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>12</v>
       </c>
@@ -4890,7 +5005,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>12</v>
       </c>
@@ -4928,7 +5043,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A91" s="8" t="s">
         <v>12</v>
       </c>
@@ -4966,7 +5081,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A92" s="8" t="s">
         <v>12</v>
       </c>
@@ -5004,7 +5119,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>12</v>
       </c>
@@ -5042,7 +5157,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>12</v>
       </c>
@@ -5080,7 +5195,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>12</v>
       </c>
@@ -5118,7 +5233,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>12</v>
       </c>
@@ -5156,7 +5271,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>12</v>
       </c>
@@ -5194,7 +5309,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>12</v>
       </c>
@@ -5232,7 +5347,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>12</v>
       </c>
@@ -5270,7 +5385,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>12</v>
       </c>
@@ -5308,7 +5423,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>12</v>
       </c>
@@ -5346,7 +5461,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>12</v>
       </c>
@@ -5384,7 +5499,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>12</v>
       </c>
@@ -5422,7 +5537,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>12</v>
       </c>
@@ -5460,7 +5575,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>12</v>
       </c>
@@ -5498,7 +5613,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>12</v>
       </c>
@@ -5536,7 +5651,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A107" s="8" t="s">
         <v>12</v>
       </c>
@@ -5574,7 +5689,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A108" s="8" t="s">
         <v>12</v>
       </c>
@@ -5612,7 +5727,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A109" s="8" t="s">
         <v>12</v>
       </c>
@@ -5650,7 +5765,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A110" s="8" t="s">
         <v>12</v>
       </c>
@@ -5688,7 +5803,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A111" s="8" t="s">
         <v>12</v>
       </c>
@@ -5726,7 +5841,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A112" s="8" t="s">
         <v>12</v>
       </c>
@@ -5764,7 +5879,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A113" s="8" t="s">
         <v>12</v>
       </c>
@@ -5802,7 +5917,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A114" s="8" t="s">
         <v>12</v>
       </c>
@@ -5840,7 +5955,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A115" s="8" t="s">
         <v>12</v>
       </c>
@@ -5878,7 +5993,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A116" s="8" t="s">
         <v>12</v>
       </c>
@@ -5916,7 +6031,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A117" s="8" t="s">
         <v>12</v>
       </c>
@@ -5954,7 +6069,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A118" s="8" t="s">
         <v>12</v>
       </c>
@@ -5992,7 +6107,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A119" s="8" t="s">
         <v>12</v>
       </c>
@@ -6030,7 +6145,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A120" s="8" t="s">
         <v>12</v>
       </c>
@@ -6068,7 +6183,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A121" s="8" t="s">
         <v>12</v>
       </c>
@@ -6106,7 +6221,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A122" s="8" t="s">
         <v>12</v>
       </c>
@@ -6144,7 +6259,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A123" s="8" t="s">
         <v>12</v>
       </c>
@@ -6182,7 +6297,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A124" s="8" t="s">
         <v>12</v>
       </c>
@@ -6220,7 +6335,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A125" s="8" t="s">
         <v>12</v>
       </c>
@@ -6258,7 +6373,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A126" s="8" t="s">
         <v>12</v>
       </c>
@@ -6296,7 +6411,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A127" s="8" t="s">
         <v>12</v>
       </c>
@@ -6334,7 +6449,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A128" s="8" t="s">
         <v>12</v>
       </c>
@@ -6372,7 +6487,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A129" s="8" t="s">
         <v>12</v>
       </c>
@@ -6410,7 +6525,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A130" s="8" t="s">
         <v>12</v>
       </c>
@@ -6448,7 +6563,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A131" s="8" t="s">
         <v>12</v>
       </c>
@@ -6486,7 +6601,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A132" s="8" t="s">
         <v>12</v>
       </c>
@@ -6524,7 +6639,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A133" s="8" t="s">
         <v>12</v>
       </c>
@@ -6562,7 +6677,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A134" s="8" t="s">
         <v>12</v>
       </c>
@@ -6600,7 +6715,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A135" s="8" t="s">
         <v>12</v>
       </c>
@@ -6638,7 +6753,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A136" s="8" t="s">
         <v>12</v>
       </c>
@@ -6676,7 +6791,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A137" s="8" t="s">
         <v>12</v>
       </c>
@@ -6714,7 +6829,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A138" s="8" t="s">
         <v>12</v>
       </c>
@@ -6752,7 +6867,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A139" s="8" t="s">
         <v>12</v>
       </c>
@@ -6790,7 +6905,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A140" s="8" t="s">
         <v>12</v>
       </c>
@@ -6828,7 +6943,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A141" s="8" t="s">
         <v>12</v>
       </c>
@@ -6866,7 +6981,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A142" s="8" t="s">
         <v>12</v>
       </c>
@@ -6904,7 +7019,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A143" s="8" t="s">
         <v>12</v>
       </c>
@@ -6950,22 +7065,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02C7B195-9C28-4152-A7C9-DCCF3DB8F404}">
   <dimension ref="A1:L44"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="21.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.77734375" customWidth="1"/>
+    <col min="2" max="2" width="21.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.83203125" customWidth="1"/>
     <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.44140625" customWidth="1"/>
-    <col min="8" max="8" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5" customWidth="1"/>
+    <col min="8" max="8" width="17.5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="25" customWidth="1"/>
-    <col min="10" max="10" width="12.21875" customWidth="1"/>
-    <col min="11" max="11" width="14.21875" customWidth="1"/>
+    <col min="10" max="10" width="12.1640625" customWidth="1"/>
+    <col min="11" max="11" width="14.1640625" customWidth="1"/>
     <col min="12" max="12" width="88" customWidth="1"/>
-    <col min="13" max="18" width="9.21875" customWidth="1"/>
+    <col min="13" max="18" width="9.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -7003,7 +7118,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -7041,7 +7156,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -7079,7 +7194,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -7117,7 +7232,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -7155,7 +7270,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -7193,7 +7308,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -7231,7 +7346,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -7269,7 +7384,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -7307,7 +7422,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -7345,7 +7460,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -7383,7 +7498,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -7421,7 +7536,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -7459,7 +7574,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -7497,7 +7612,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -7535,7 +7650,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>12</v>
       </c>
@@ -7573,7 +7688,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>12</v>
       </c>
@@ -7611,7 +7726,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>12</v>
       </c>
@@ -7649,7 +7764,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>12</v>
       </c>
@@ -7687,7 +7802,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -7725,7 +7840,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>12</v>
       </c>
@@ -7763,7 +7878,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>12</v>
       </c>
@@ -7801,7 +7916,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>12</v>
       </c>
@@ -7839,7 +7954,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>12</v>
       </c>
@@ -7877,7 +7992,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -7915,7 +8030,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>12</v>
       </c>
@@ -7953,7 +8068,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>12</v>
       </c>
@@ -7991,7 +8106,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>12</v>
       </c>
@@ -8029,7 +8144,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>12</v>
       </c>
@@ -8067,7 +8182,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>12</v>
       </c>
@@ -8105,7 +8220,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>12</v>
       </c>
@@ -8143,7 +8258,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>12</v>
       </c>
@@ -8181,7 +8296,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>12</v>
       </c>
@@ -8219,7 +8334,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>12</v>
       </c>
@@ -8257,7 +8372,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>12</v>
       </c>
@@ -8295,7 +8410,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>12</v>
       </c>
@@ -8333,7 +8448,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>12</v>
       </c>
@@ -8371,7 +8486,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>12</v>
       </c>
@@ -8409,7 +8524,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>12</v>
       </c>
@@ -8447,7 +8562,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>12</v>
       </c>
@@ -8485,7 +8600,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>12</v>
       </c>
@@ -8523,7 +8638,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>12</v>
       </c>
@@ -8561,7 +8676,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>12</v>
       </c>
@@ -8599,7 +8714,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>12</v>
       </c>
@@ -8645,21 +8760,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA328016-6EE1-4F6F-84C5-5395FF87B11C}">
   <dimension ref="A1:L43"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="52.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.21875" customWidth="1"/>
-    <col min="6" max="6" width="10.5546875" customWidth="1"/>
-    <col min="7" max="7" width="14.21875" customWidth="1"/>
-    <col min="8" max="8" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.21875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="93.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="52.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.1640625" customWidth="1"/>
+    <col min="6" max="6" width="10.5" customWidth="1"/>
+    <col min="7" max="7" width="14.1640625" customWidth="1"/>
+    <col min="8" max="8" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="93.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -8697,7 +8812,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -8735,7 +8850,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -8773,7 +8888,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -8811,7 +8926,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -8849,7 +8964,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -8887,7 +9002,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -8925,7 +9040,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -8963,7 +9078,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -9001,7 +9116,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -9039,7 +9154,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -9077,7 +9192,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -9115,7 +9230,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -9153,7 +9268,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -9191,7 +9306,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -9229,7 +9344,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>12</v>
       </c>
@@ -9267,7 +9382,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>12</v>
       </c>
@@ -9305,7 +9420,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>12</v>
       </c>
@@ -9343,7 +9458,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>12</v>
       </c>
@@ -9381,7 +9496,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -9419,7 +9534,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>12</v>
       </c>
@@ -9457,7 +9572,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>12</v>
       </c>
@@ -9495,7 +9610,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>12</v>
       </c>
@@ -9533,7 +9648,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>12</v>
       </c>
@@ -9571,7 +9686,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -9609,7 +9724,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>12</v>
       </c>
@@ -9647,7 +9762,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>12</v>
       </c>
@@ -9685,7 +9800,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>12</v>
       </c>
@@ -9723,7 +9838,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>12</v>
       </c>
@@ -9761,7 +9876,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>12</v>
       </c>
@@ -9799,7 +9914,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>12</v>
       </c>
@@ -9837,7 +9952,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>12</v>
       </c>
@@ -9875,7 +9990,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>12</v>
       </c>
@@ -9913,7 +10028,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>12</v>
       </c>
@@ -9951,7 +10066,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>12</v>
       </c>
@@ -9989,7 +10104,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>12</v>
       </c>
@@ -10027,7 +10142,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>12</v>
       </c>
@@ -10065,7 +10180,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>12</v>
       </c>
@@ -10103,7 +10218,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>12</v>
       </c>
@@ -10141,7 +10256,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>12</v>
       </c>
@@ -10179,7 +10294,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>12</v>
       </c>
@@ -10217,7 +10332,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>12</v>
       </c>
@@ -10255,7 +10370,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>12</v>
       </c>
@@ -10301,18 +10416,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E6501C2-1F4E-44C1-926E-7B80FAB5E9FA}">
   <dimension ref="A1:L22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="38" customWidth="1"/>
-    <col min="5" max="5" width="22.77734375" customWidth="1"/>
-    <col min="8" max="8" width="18.77734375" customWidth="1"/>
-    <col min="9" max="9" width="14.77734375" customWidth="1"/>
-    <col min="10" max="10" width="18.5546875" customWidth="1"/>
-    <col min="11" max="11" width="15.77734375" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.5" customWidth="1"/>
+    <col min="11" max="11" width="15.83203125" customWidth="1"/>
     <col min="12" max="12" width="54" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -10350,7 +10465,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -10388,7 +10503,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -10426,7 +10541,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -10464,7 +10579,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -10502,7 +10617,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
         <v>12</v>
       </c>
@@ -10540,7 +10655,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
         <v>12</v>
       </c>
@@ -10578,7 +10693,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -10616,7 +10731,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -10654,7 +10769,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -10692,7 +10807,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -10730,7 +10845,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -10768,7 +10883,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -10806,7 +10921,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -10844,7 +10959,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -10882,7 +10997,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>12</v>
       </c>
@@ -10920,7 +11035,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>12</v>
       </c>
@@ -10958,7 +11073,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>12</v>
       </c>
@@ -10996,7 +11111,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>12</v>
       </c>
@@ -11034,7 +11149,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -11072,7 +11187,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>12</v>
       </c>
@@ -11110,7 +11225,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="L22" s="19"/>
     </row>
   </sheetData>
@@ -11121,16 +11236,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CE0DD1A-FCA4-41B6-815F-1DF4FD2DD0A1}">
   <dimension ref="A1:L46"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="10.77734375" customWidth="1"/>
-    <col min="3" max="3" width="9.21875" customWidth="1"/>
-    <col min="4" max="4" width="38.5546875" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="9.1640625" customWidth="1"/>
+    <col min="4" max="4" width="38.5" customWidth="1"/>
     <col min="5" max="12" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -11168,7 +11283,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
         <v>12</v>
       </c>
@@ -11206,7 +11321,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
         <v>12</v>
       </c>
@@ -11244,7 +11359,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
         <v>12</v>
       </c>
@@ -11282,7 +11397,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
         <v>12</v>
       </c>
@@ -11320,7 +11435,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
         <v>12</v>
       </c>
@@ -11358,7 +11473,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
         <v>12</v>
       </c>
@@ -11396,7 +11511,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>12</v>
       </c>
@@ -11434,7 +11549,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
         <v>12</v>
       </c>
@@ -11472,7 +11587,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
         <v>12</v>
       </c>
@@ -11510,7 +11625,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="8" t="s">
         <v>12</v>
       </c>
@@ -11548,7 +11663,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="8" t="s">
         <v>12</v>
       </c>
@@ -11586,7 +11701,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="8" t="s">
         <v>12</v>
       </c>
@@ -11624,7 +11739,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="8" t="s">
         <v>12</v>
       </c>
@@ -11662,7 +11777,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="8" t="s">
         <v>12</v>
       </c>
@@ -11700,7 +11815,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="8" t="s">
         <v>12</v>
       </c>
@@ -11738,7 +11853,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
         <v>12</v>
       </c>
@@ -11776,7 +11891,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="8" t="s">
         <v>12</v>
       </c>
@@ -11814,7 +11929,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="8" t="s">
         <v>12</v>
       </c>
@@ -11852,7 +11967,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="8" t="s">
         <v>12</v>
       </c>
@@ -11890,7 +12005,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="8" t="s">
         <v>12</v>
       </c>
@@ -11928,7 +12043,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="8" t="s">
         <v>12</v>
       </c>
@@ -11966,7 +12081,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="8" t="s">
         <v>12</v>
       </c>
@@ -12004,7 +12119,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="8" t="s">
         <v>12</v>
       </c>
@@ -12042,7 +12157,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="8" t="s">
         <v>12</v>
       </c>
@@ -12080,7 +12195,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="8" t="s">
         <v>12</v>
       </c>
@@ -12118,7 +12233,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="8" t="s">
         <v>12</v>
       </c>
@@ -12156,7 +12271,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="8" t="s">
         <v>12</v>
       </c>
@@ -12194,7 +12309,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="8" t="s">
         <v>12</v>
       </c>
@@ -12232,7 +12347,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="8" t="s">
         <v>12</v>
       </c>
@@ -12270,7 +12385,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" s="8" t="s">
         <v>12</v>
       </c>
@@ -12308,7 +12423,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" s="8" t="s">
         <v>12</v>
       </c>
@@ -12346,7 +12461,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" s="8" t="s">
         <v>12</v>
       </c>
@@ -12384,7 +12499,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" s="8" t="s">
         <v>12</v>
       </c>
@@ -12422,7 +12537,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" s="8" t="s">
         <v>12</v>
       </c>
@@ -12460,7 +12575,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" s="8" t="s">
         <v>12</v>
       </c>
@@ -12498,7 +12613,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" s="8" t="s">
         <v>12</v>
       </c>
@@ -12536,7 +12651,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" s="8" t="s">
         <v>12</v>
       </c>
@@ -12574,29 +12689,577 @@
         <v>310</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="D39" s="14"/>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="D40" s="14"/>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="D41" s="14"/>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="D42" s="14"/>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="D43" s="14"/>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="D44" s="14"/>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="D45" s="15"/>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="D46" s="15"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2977C247-05DC-724D-A00A-EDAB54DF4626}">
+  <dimension ref="A1:L15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="19" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="33.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="59.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>262</v>
+      </c>
+      <c r="D2" t="s">
+        <v>316</v>
+      </c>
+      <c r="E2" t="s">
+        <v>317</v>
+      </c>
+      <c r="F2" t="s">
+        <v>62</v>
+      </c>
+      <c r="G2" t="s">
+        <v>86</v>
+      </c>
+      <c r="H2" t="s">
+        <v>100</v>
+      </c>
+      <c r="I2" t="s">
+        <v>318</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="K2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L2" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>262</v>
+      </c>
+      <c r="D3" t="s">
+        <v>320</v>
+      </c>
+      <c r="E3" t="s">
+        <v>321</v>
+      </c>
+      <c r="F3" t="s">
+        <v>62</v>
+      </c>
+      <c r="G3" t="s">
+        <v>78</v>
+      </c>
+      <c r="H3" t="s">
+        <v>100</v>
+      </c>
+      <c r="I3" t="s">
+        <v>322</v>
+      </c>
+      <c r="J3" t="s">
+        <v>80</v>
+      </c>
+      <c r="K3" t="s">
+        <v>81</v>
+      </c>
+      <c r="L3" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>262</v>
+      </c>
+      <c r="D4" t="s">
+        <v>324</v>
+      </c>
+      <c r="E4" t="s">
+        <v>321</v>
+      </c>
+      <c r="F4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G4" t="s">
+        <v>325</v>
+      </c>
+      <c r="H4" t="s">
+        <v>100</v>
+      </c>
+      <c r="I4" t="s">
+        <v>326</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="K4" t="s">
+        <v>157</v>
+      </c>
+      <c r="L4" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>262</v>
+      </c>
+      <c r="D5" t="s">
+        <v>328</v>
+      </c>
+      <c r="E5" t="s">
+        <v>321</v>
+      </c>
+      <c r="F5" t="s">
+        <v>62</v>
+      </c>
+      <c r="G5" t="s">
+        <v>86</v>
+      </c>
+      <c r="H5" t="s">
+        <v>79</v>
+      </c>
+      <c r="I5" t="s">
+        <v>326</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="K5" t="s">
+        <v>81</v>
+      </c>
+      <c r="L5" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>262</v>
+      </c>
+      <c r="D6" t="s">
+        <v>330</v>
+      </c>
+      <c r="E6" t="s">
+        <v>321</v>
+      </c>
+      <c r="F6" t="s">
+        <v>62</v>
+      </c>
+      <c r="G6" t="s">
+        <v>86</v>
+      </c>
+      <c r="H6" t="s">
+        <v>79</v>
+      </c>
+      <c r="I6" t="s">
+        <v>326</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="K6" t="s">
+        <v>81</v>
+      </c>
+      <c r="L6" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>262</v>
+      </c>
+      <c r="D7" t="s">
+        <v>332</v>
+      </c>
+      <c r="E7" t="s">
+        <v>321</v>
+      </c>
+      <c r="F7" t="s">
+        <v>62</v>
+      </c>
+      <c r="G7" t="s">
+        <v>86</v>
+      </c>
+      <c r="H7" t="s">
+        <v>100</v>
+      </c>
+      <c r="I7" t="s">
+        <v>326</v>
+      </c>
+      <c r="J7" t="s">
+        <v>80</v>
+      </c>
+      <c r="K7" t="s">
+        <v>81</v>
+      </c>
+      <c r="L7" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>262</v>
+      </c>
+      <c r="D8" t="s">
+        <v>334</v>
+      </c>
+      <c r="E8" t="s">
+        <v>321</v>
+      </c>
+      <c r="F8" t="s">
+        <v>68</v>
+      </c>
+      <c r="G8" t="s">
+        <v>86</v>
+      </c>
+      <c r="H8" t="s">
+        <v>79</v>
+      </c>
+      <c r="I8" t="s">
+        <v>326</v>
+      </c>
+      <c r="J8" t="s">
+        <v>80</v>
+      </c>
+      <c r="K8" t="s">
+        <v>81</v>
+      </c>
+      <c r="L8" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>262</v>
+      </c>
+      <c r="D9" t="s">
+        <v>336</v>
+      </c>
+      <c r="E9" t="s">
+        <v>321</v>
+      </c>
+      <c r="F9" t="s">
+        <v>62</v>
+      </c>
+      <c r="G9" t="s">
+        <v>78</v>
+      </c>
+      <c r="H9" t="s">
+        <v>100</v>
+      </c>
+      <c r="I9" t="s">
+        <v>326</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="K9" t="s">
+        <v>81</v>
+      </c>
+      <c r="L9" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
+        <v>262</v>
+      </c>
+      <c r="D10" t="s">
+        <v>338</v>
+      </c>
+      <c r="E10" t="s">
+        <v>321</v>
+      </c>
+      <c r="F10" t="s">
+        <v>15</v>
+      </c>
+      <c r="G10" t="s">
+        <v>339</v>
+      </c>
+      <c r="H10" t="s">
+        <v>79</v>
+      </c>
+      <c r="I10" t="s">
+        <v>340</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="K10" t="s">
+        <v>157</v>
+      </c>
+      <c r="L10" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>262</v>
+      </c>
+      <c r="D11" t="s">
+        <v>342</v>
+      </c>
+      <c r="E11" t="s">
+        <v>321</v>
+      </c>
+      <c r="F11" t="s">
+        <v>15</v>
+      </c>
+      <c r="G11" t="s">
+        <v>78</v>
+      </c>
+      <c r="H11" t="s">
+        <v>100</v>
+      </c>
+      <c r="I11" t="s">
+        <v>322</v>
+      </c>
+      <c r="J11" t="s">
+        <v>80</v>
+      </c>
+      <c r="K11" t="s">
+        <v>81</v>
+      </c>
+      <c r="L11" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>262</v>
+      </c>
+      <c r="D12" t="s">
+        <v>344</v>
+      </c>
+      <c r="E12" t="s">
+        <v>321</v>
+      </c>
+      <c r="F12" t="s">
+        <v>62</v>
+      </c>
+      <c r="G12" t="s">
+        <v>130</v>
+      </c>
+      <c r="H12" t="s">
+        <v>100</v>
+      </c>
+      <c r="I12" t="s">
+        <v>326</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="K12" t="s">
+        <v>81</v>
+      </c>
+      <c r="L12" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>262</v>
+      </c>
+      <c r="D13" t="s">
+        <v>346</v>
+      </c>
+      <c r="E13" t="s">
+        <v>321</v>
+      </c>
+      <c r="F13" t="s">
+        <v>62</v>
+      </c>
+      <c r="G13" t="s">
+        <v>130</v>
+      </c>
+      <c r="H13" t="s">
+        <v>100</v>
+      </c>
+      <c r="I13" t="s">
+        <v>347</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="K13" t="s">
+        <v>81</v>
+      </c>
+      <c r="L13" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>262</v>
+      </c>
+      <c r="D14" t="s">
+        <v>349</v>
+      </c>
+      <c r="E14" t="s">
+        <v>321</v>
+      </c>
+      <c r="F14" t="s">
+        <v>62</v>
+      </c>
+      <c r="G14" t="s">
+        <v>130</v>
+      </c>
+      <c r="H14" t="s">
+        <v>100</v>
+      </c>
+      <c r="I14" t="s">
+        <v>347</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="K14" t="s">
+        <v>81</v>
+      </c>
+      <c r="L14" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" t="s">
+        <v>262</v>
+      </c>
+      <c r="D15" t="s">
+        <v>351</v>
+      </c>
+      <c r="E15" t="s">
+        <v>352</v>
+      </c>
+      <c r="F15" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" t="s">
+        <v>127</v>
+      </c>
+      <c r="H15" t="s">
+        <v>100</v>
+      </c>
+      <c r="I15" t="s">
+        <v>322</v>
+      </c>
+      <c r="J15" t="s">
+        <v>80</v>
+      </c>
+      <c r="K15" t="s">
+        <v>81</v>
+      </c>
+      <c r="L15" t="s">
+        <v>353</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>